<commit_message>
Merge Gulf deep gap-fill outputs into Saudi, UAE, Qatar, Kuwait prospect workbooks
Add merge_gap_outputs.py (dedupe by store URL and (store, person), fill-only
contact merge, LinkedIn corrections) and regenerate the 8 Gulf workbooks.

Co-authored-by: abaszeinn-beep <abaszeinn-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/markets/prospects/Kuwait_Fashion_Prospects.xlsx
+++ b/markets/prospects/Kuwait_Fashion_Prospects.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Prospects'!$A$1:$J$61</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Decision Makers'!$A$1:$G$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Decision Makers'!$A$1:$G$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2732,12 +2732,12 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Amir Al-Hinnawi</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Managing Partner, Starco Holding; CEO Bevava (e-commerce)</t>
         </is>
       </c>
     </row>
@@ -3266,12 +3266,12 @@
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Micheline Berzy</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Head of Marketing - Fashion Brands (incl. Ted Baker), Al-Futtaim</t>
         </is>
       </c>
     </row>
@@ -3362,12 +3362,12 @@
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Sarah N. AlThekair</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Co-Founder &amp; CEO</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>+965 55041174</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -3597,7 +3597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G98"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7016,22 +7016,22 @@
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>Styli</t>
+          <t>U.S. Polo Assn. Kuwait</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>https://stylishop.com/kw/en</t>
+          <t>https://www.uspoloassn.com.kw/</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Shibu Tharakan</t>
+          <t>Amir Al-Hinnawi</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>Chief Executive Officer, Styli (Landmark Group)</t>
+          <t>Managing Partner Kuwait &amp; Lebanon, Starco Holding; CEO, Bevava (e-commerce platform for Starco franchised brands)</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -7046,29 +7046,29 @@
       </c>
       <c r="G93" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/shibutharakan</t>
+          <t>https://linkedin.com/in/amiralhinnawi</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Thoubi</t>
+          <t>U.S. Polo Assn. Kuwait</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>https://thoubi.com/</t>
+          <t>https://www.uspoloassn.com.kw/</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Nabil Ahmed</t>
+          <t>Mohamad Hadi</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Head Of Ecommerce at Thoubi.com</t>
+          <t>Brands Manager (U.S. Polo Assn., Benetton, Eden Park), Starco Holding</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -7083,29 +7083,29 @@
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/nabil-ahmed-93265b114</t>
+          <t>https://linkedin.com/in/mohamad-hadi-140730a0</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>Squatwolf Kuwait (AAW franchise)</t>
+          <t>U.S. Polo Assn. Kuwait</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>https://squatwolf.com/en-kw/</t>
+          <t>https://www.uspoloassn.com.kw/</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Louay Baalbaky</t>
+          <t>Jamal Al-Hinnawi</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>Sr. Brand Manager - Intersport &amp; Squatwolf (Kuwait), AAW</t>
+          <t>President &amp; CEO, Starco Holding</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -7120,29 +7120,29 @@
       </c>
       <c r="G95" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/louay-baalbaky-47626b29</t>
+          <t>https://linkedin.com/in/jamal-al-hinnawi-1ba8619</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Squatwolf Kuwait (AAW franchise)</t>
+          <t>Styli</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>https://squatwolf.com/en-kw/</t>
+          <t>https://stylishop.com/kw/en</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Murtaza Fakhruddin</t>
+          <t>Shibu Tharakan</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Senior Projects Manager - Ecommerce, Ali Abdulwahab Al Mutawa Commercial Co. (AAW) (LinkedIn headline; experience entry still lists Head of Ecommerce since Mar 2020)</t>
+          <t>Chief Executive Officer, Styli (Landmark Group)</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -7157,29 +7157,29 @@
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/murtaza-fakhruddin-0692681b</t>
+          <t>https://www.linkedin.com/in/shibutharakan</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>Squatwolf Kuwait (AAW franchise)</t>
+          <t>Thoubi</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>https://squatwolf.com/en-kw/</t>
+          <t>https://thoubi.com/</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Hala Thiab</t>
+          <t>Nabil Ahmed</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>Senior eCommerce Manager, Ali Abdulwahab Al Mutawa Commercial Co. (AAW) (Sep 2020-present)</t>
+          <t>Head Of Ecommerce at Thoubi.com</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -7194,49 +7194,271 @@
       </c>
       <c r="G97" s="6" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/hala-thiab-44a60956</t>
+          <t>https://www.linkedin.com/in/nabil-ahmed-93265b114</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
+          <t>Ted Baker KW</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tedbaker.kw/</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Micheline Berzy</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Head of Marketing - Fashion Brands (Sandro, Maje, Claudie Pierlot, Ted Baker), Al-Futtaim</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/michelineberzy</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>Ted Baker KW</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>https://www.tedbaker.kw/</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Sanja Gorgieva</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>Regional Brand Manager - Ted Baker (MENA), Al-Futtaim</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G99" s="6" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/sanja-gorgieva-b912a087</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Squatwolf Kuwait (AAW franchise)</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>https://squatwolf.com/en-kw/</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Louay Baalbaky</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Sr. Brand Manager - Intersport &amp; Squatwolf (Kuwait), AAW</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/louay-baalbaky-47626b29</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>Squatwolf Kuwait (AAW franchise)</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>https://squatwolf.com/en-kw/</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Murtaza Fakhruddin</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>Senior Projects Manager - Ecommerce, Ali Abdulwahab Al Mutawa Commercial Co. (AAW) (LinkedIn headline; experience entry still lists Head of Ecommerce since Mar 2020)</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G101" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/murtaza-fakhruddin-0692681b</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Squatwolf Kuwait (AAW franchise)</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>https://squatwolf.com/en-kw/</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Hala Thiab</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Senior eCommerce Manager, Ali Abdulwahab Al Mutawa Commercial Co. (AAW) (Sep 2020-present)</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/hala-thiab-44a60956</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>Modish</t>
+        </is>
+      </c>
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>https://modish.com.kw/</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Sarah N. AlThekair</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
           <t>aivi</t>
         </is>
       </c>
-      <c r="B98" s="3" t="inlineStr">
+      <c r="B104" s="3" t="inlineStr">
         <is>
           <t>https://en-kw.aivi.com/</t>
         </is>
       </c>
-      <c r="C98" s="2" t="inlineStr">
+      <c r="C104" s="2" t="inlineStr">
         <is>
           <t>Vivek Rajukumar</t>
         </is>
       </c>
-      <c r="D98" s="2" t="inlineStr">
+      <c r="D104" s="2" t="inlineStr">
         <is>
           <t>Chief Executive Officer, AIVI (formerly 6thStreet, Apparel Group)</t>
         </is>
       </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="F98" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="G98" s="3" t="inlineStr">
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G104" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/vivek-rajukumar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G98"/>
+  <autoFilter ref="A1:G104"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -7429,6 +7651,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B99" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B100" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B101" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="rId202"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>